<commit_message>
Ajuste do Grafico de Gannt
</commit_message>
<xml_diff>
--- a/docs/Gráfico de Gantt.xlsx
+++ b/docs/Gráfico de Gantt.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="38">
   <si>
     <t xml:space="preserve">Atividade</t>
   </si>
@@ -49,7 +49,7 @@
     <t xml:space="preserve">Sprint 8</t>
   </si>
   <si>
-    <t xml:space="preserve">Sprint 9</t>
+    <t xml:space="preserve">Sprint 9(Q.A)</t>
   </si>
   <si>
     <t xml:space="preserve">Sprint 10</t>
@@ -95,6 +95,45 @@
   </si>
   <si>
     <t xml:space="preserve">CRUD professores</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Modelo conceitual do banco (DER)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Diagrama de caso de uso</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Diagrama de classes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Arquitetura de software</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Escolha da stack</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Proposta de solução</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Organização da equipe</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Definição de papéis</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Apresentação e deploy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Documentação final</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ajustes requisitados pela organização</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Apresentação publica</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Distribuição do link ao público geral</t>
   </si>
 </sst>
 </file>
@@ -198,7 +237,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -208,19 +247,15 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -480,7 +515,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="25" min="12" style="1" width="8.71"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -515,183 +550,183 @@
         <v>10</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="B2" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="C2" s="4"/>
-      <c r="D2" s="4"/>
-      <c r="E2" s="4"/>
-      <c r="F2" s="4"/>
-      <c r="G2" s="4"/>
-      <c r="H2" s="4"/>
-      <c r="I2" s="4"/>
-      <c r="J2" s="4"/>
-      <c r="K2" s="4"/>
+      <c r="B2" s="3"/>
+      <c r="C2" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="D2" s="3"/>
+      <c r="E2" s="3"/>
+      <c r="F2" s="3"/>
+      <c r="G2" s="3"/>
+      <c r="H2" s="3"/>
+      <c r="I2" s="3"/>
+      <c r="J2" s="3"/>
+      <c r="K2" s="3"/>
     </row>
     <row r="3" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="5" t="s">
+      <c r="A3" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="B3" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="C3" s="4"/>
-      <c r="D3" s="4"/>
-      <c r="E3" s="4"/>
-      <c r="F3" s="4"/>
-      <c r="G3" s="4"/>
-      <c r="H3" s="4"/>
-      <c r="I3" s="4"/>
-      <c r="J3" s="4"/>
-      <c r="K3" s="4"/>
+      <c r="B3" s="3"/>
+      <c r="C3" s="3"/>
+      <c r="D3" s="3"/>
+      <c r="E3" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F3" s="3"/>
+      <c r="G3" s="3"/>
+      <c r="H3" s="3"/>
+      <c r="I3" s="3"/>
+      <c r="J3" s="3"/>
+      <c r="K3" s="3"/>
     </row>
     <row r="4" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="4" t="s">
+      <c r="A4" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="B4" s="4"/>
-      <c r="C4" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="D4" s="4"/>
-      <c r="E4" s="4"/>
-      <c r="F4" s="4"/>
-      <c r="G4" s="4"/>
-      <c r="H4" s="4"/>
-      <c r="I4" s="4"/>
-      <c r="J4" s="4"/>
-      <c r="K4" s="4"/>
+      <c r="B4" s="3"/>
+      <c r="C4" s="3"/>
+      <c r="D4" s="3"/>
+      <c r="E4" s="3"/>
+      <c r="F4" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G4" s="3"/>
+      <c r="H4" s="3"/>
+      <c r="I4" s="3"/>
+      <c r="J4" s="3"/>
+      <c r="K4" s="3"/>
     </row>
     <row r="5" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="4" t="s">
+      <c r="A5" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="B5" s="4"/>
-      <c r="C5" s="4"/>
-      <c r="D5" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="E5" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="F5" s="4"/>
-      <c r="G5" s="4"/>
-      <c r="H5" s="4"/>
-      <c r="I5" s="4"/>
-      <c r="J5" s="4"/>
-      <c r="K5" s="4"/>
+      <c r="B5" s="3"/>
+      <c r="C5" s="3"/>
+      <c r="D5" s="3"/>
+      <c r="E5" s="3"/>
+      <c r="F5" s="3"/>
+      <c r="G5" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="H5" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="I5" s="3"/>
+      <c r="J5" s="3"/>
+      <c r="K5" s="3"/>
     </row>
     <row r="6" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="4" t="s">
+      <c r="A6" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="B6" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="C6" s="4"/>
-      <c r="D6" s="4"/>
-      <c r="E6" s="4"/>
-      <c r="F6" s="4"/>
-      <c r="G6" s="4"/>
-      <c r="H6" s="4"/>
-      <c r="I6" s="4"/>
-      <c r="J6" s="4"/>
-      <c r="K6" s="4"/>
+      <c r="B6" s="3"/>
+      <c r="C6" s="3"/>
+      <c r="D6" s="3"/>
+      <c r="E6" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F6" s="3"/>
+      <c r="G6" s="3"/>
+      <c r="H6" s="3"/>
+      <c r="I6" s="3"/>
+      <c r="J6" s="3"/>
+      <c r="K6" s="3"/>
     </row>
     <row r="7" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="4" t="s">
+      <c r="A7" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="B7" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="C7" s="4"/>
-      <c r="D7" s="4"/>
-      <c r="E7" s="4"/>
-      <c r="F7" s="4"/>
-      <c r="G7" s="4"/>
-      <c r="H7" s="4"/>
-      <c r="I7" s="4"/>
-      <c r="J7" s="4"/>
-      <c r="K7" s="4"/>
+      <c r="B7" s="3"/>
+      <c r="C7" s="3"/>
+      <c r="D7" s="3"/>
+      <c r="E7" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F7" s="3"/>
+      <c r="G7" s="3"/>
+      <c r="H7" s="3"/>
+      <c r="I7" s="3"/>
+      <c r="J7" s="3"/>
+      <c r="K7" s="3"/>
     </row>
     <row r="8" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="4" t="s">
+      <c r="A8" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="B8" s="4"/>
-      <c r="C8" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="D8" s="4"/>
-      <c r="E8" s="4"/>
-      <c r="F8" s="4"/>
-      <c r="G8" s="4"/>
-      <c r="H8" s="4"/>
-      <c r="I8" s="4"/>
-      <c r="J8" s="4"/>
-      <c r="K8" s="4"/>
+      <c r="B8" s="3"/>
+      <c r="C8" s="3"/>
+      <c r="D8" s="3"/>
+      <c r="E8" s="3"/>
+      <c r="F8" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G8" s="3"/>
+      <c r="H8" s="3"/>
+      <c r="I8" s="3"/>
+      <c r="J8" s="3"/>
+      <c r="K8" s="3"/>
     </row>
     <row r="9" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="4" t="s">
+      <c r="A9" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="B9" s="4"/>
-      <c r="C9" s="4"/>
-      <c r="D9" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="E9" s="4"/>
-      <c r="F9" s="4"/>
-      <c r="G9" s="4"/>
-      <c r="H9" s="4"/>
-      <c r="I9" s="4"/>
-      <c r="J9" s="4"/>
-      <c r="K9" s="4"/>
+      <c r="B9" s="3"/>
+      <c r="C9" s="3"/>
+      <c r="D9" s="3"/>
+      <c r="E9" s="3"/>
+      <c r="F9" s="3"/>
+      <c r="G9" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="H9" s="3"/>
+      <c r="I9" s="3"/>
+      <c r="J9" s="3"/>
+      <c r="K9" s="3"/>
     </row>
     <row r="10" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="4" t="s">
+      <c r="A10" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="B10" s="4"/>
-      <c r="C10" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="D10" s="4"/>
-      <c r="E10" s="4"/>
-      <c r="F10" s="4"/>
-      <c r="G10" s="4"/>
-      <c r="H10" s="4"/>
-      <c r="I10" s="4"/>
-      <c r="J10" s="4"/>
-      <c r="K10" s="4"/>
+      <c r="B10" s="3"/>
+      <c r="C10" s="3"/>
+      <c r="D10" s="3"/>
+      <c r="E10" s="3"/>
+      <c r="F10" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G10" s="3"/>
+      <c r="H10" s="3"/>
+      <c r="I10" s="3"/>
+      <c r="J10" s="3"/>
+      <c r="K10" s="3"/>
     </row>
     <row r="11" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="4" t="s">
+      <c r="A11" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="B11" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="C11" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="D11" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="E11" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="F11" s="4"/>
-      <c r="G11" s="4"/>
-      <c r="H11" s="4"/>
-      <c r="I11" s="4"/>
-      <c r="J11" s="4"/>
-      <c r="K11" s="4"/>
+      <c r="B11" s="3"/>
+      <c r="C11" s="3"/>
+      <c r="D11" s="3"/>
+      <c r="E11" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F11" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G11" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="H11" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="I11" s="3"/>
+      <c r="J11" s="3"/>
+      <c r="K11" s="3"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="3" t="s">
@@ -700,12 +735,12 @@
       <c r="B12" s="3"/>
       <c r="C12" s="3"/>
       <c r="D12" s="3"/>
-      <c r="E12" s="3" t="s">
-        <v>12</v>
-      </c>
+      <c r="E12" s="3"/>
       <c r="F12" s="3"/>
       <c r="G12" s="3"/>
-      <c r="H12" s="3"/>
+      <c r="H12" s="3" t="s">
+        <v>12</v>
+      </c>
       <c r="I12" s="3"/>
       <c r="J12" s="3"/>
       <c r="K12" s="3"/>
@@ -717,40 +752,266 @@
       <c r="B13" s="3"/>
       <c r="C13" s="3"/>
       <c r="D13" s="3"/>
-      <c r="E13" s="3" t="s">
-        <v>12</v>
-      </c>
+      <c r="E13" s="3"/>
       <c r="F13" s="3"/>
       <c r="G13" s="3"/>
-      <c r="H13" s="3"/>
+      <c r="H13" s="3" t="s">
+        <v>12</v>
+      </c>
       <c r="I13" s="3"/>
       <c r="J13" s="3"/>
       <c r="K13" s="3"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="4" t="s">
+      <c r="A14" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="B14" s="4"/>
-      <c r="C14" s="4"/>
-      <c r="D14" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="E14" s="4"/>
-      <c r="F14" s="4"/>
-      <c r="G14" s="4"/>
-      <c r="H14" s="4"/>
-      <c r="I14" s="4"/>
-      <c r="J14" s="4"/>
-      <c r="K14" s="4"/>
-    </row>
-    <row r="21" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="22" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="23" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="24" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="25" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="26" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="27" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+      <c r="B14" s="3"/>
+      <c r="C14" s="3"/>
+      <c r="D14" s="3"/>
+      <c r="E14" s="3"/>
+      <c r="F14" s="3"/>
+      <c r="G14" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="H14" s="3"/>
+      <c r="I14" s="3"/>
+      <c r="J14" s="3"/>
+      <c r="K14" s="3"/>
+    </row>
+    <row r="15" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="B15" s="3"/>
+      <c r="C15" s="3"/>
+      <c r="D15" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E15" s="3"/>
+      <c r="F15" s="3"/>
+      <c r="G15" s="3"/>
+      <c r="H15" s="3"/>
+      <c r="I15" s="3"/>
+      <c r="J15" s="3"/>
+      <c r="K15" s="3"/>
+    </row>
+    <row r="16" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="B16" s="3"/>
+      <c r="C16" s="3"/>
+      <c r="D16" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E16" s="3"/>
+      <c r="F16" s="3"/>
+      <c r="G16" s="3"/>
+      <c r="H16" s="3"/>
+      <c r="I16" s="3"/>
+      <c r="J16" s="3"/>
+      <c r="K16" s="3"/>
+    </row>
+    <row r="17" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="B17" s="3"/>
+      <c r="C17" s="3"/>
+      <c r="D17" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E17" s="3"/>
+      <c r="F17" s="3"/>
+      <c r="G17" s="3"/>
+      <c r="H17" s="3"/>
+      <c r="I17" s="3"/>
+      <c r="J17" s="3"/>
+      <c r="K17" s="3"/>
+    </row>
+    <row r="18" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="B18" s="3"/>
+      <c r="C18" s="3"/>
+      <c r="D18" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E18" s="3"/>
+      <c r="F18" s="3"/>
+      <c r="G18" s="3"/>
+      <c r="H18" s="3"/>
+      <c r="I18" s="3"/>
+      <c r="J18" s="3"/>
+      <c r="K18" s="3"/>
+    </row>
+    <row r="19" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="B19" s="3"/>
+      <c r="C19" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="D19" s="3"/>
+      <c r="E19" s="3"/>
+      <c r="F19" s="3"/>
+      <c r="G19" s="3"/>
+      <c r="H19" s="3"/>
+      <c r="I19" s="3"/>
+      <c r="J19" s="3"/>
+      <c r="K19" s="3"/>
+    </row>
+    <row r="20" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="B20" s="3"/>
+      <c r="C20" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="D20" s="3"/>
+      <c r="E20" s="3"/>
+      <c r="F20" s="3"/>
+      <c r="G20" s="3"/>
+      <c r="H20" s="3"/>
+      <c r="I20" s="3"/>
+      <c r="J20" s="3"/>
+      <c r="K20" s="3"/>
+    </row>
+    <row r="21" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="B21" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C21" s="3"/>
+      <c r="D21" s="3"/>
+      <c r="E21" s="3"/>
+      <c r="F21" s="3"/>
+      <c r="G21" s="3"/>
+      <c r="H21" s="3"/>
+      <c r="I21" s="3"/>
+      <c r="J21" s="3"/>
+      <c r="K21" s="3"/>
+    </row>
+    <row r="22" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="B22" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C22" s="3"/>
+      <c r="D22" s="3"/>
+      <c r="E22" s="3"/>
+      <c r="F22" s="3"/>
+      <c r="G22" s="3"/>
+      <c r="H22" s="3"/>
+      <c r="I22" s="3"/>
+      <c r="J22" s="3"/>
+      <c r="K22" s="3"/>
+    </row>
+    <row r="23" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="B23" s="3"/>
+      <c r="C23" s="3"/>
+      <c r="D23" s="3"/>
+      <c r="E23" s="3"/>
+      <c r="F23" s="3"/>
+      <c r="G23" s="3"/>
+      <c r="H23" s="3"/>
+      <c r="I23" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="J23" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="K23" s="3" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="B24" s="3"/>
+      <c r="C24" s="3"/>
+      <c r="D24" s="3"/>
+      <c r="E24" s="3"/>
+      <c r="F24" s="3"/>
+      <c r="G24" s="3"/>
+      <c r="H24" s="3"/>
+      <c r="I24" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="J24" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="K24" s="3" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="B25" s="3"/>
+      <c r="C25" s="3"/>
+      <c r="D25" s="3"/>
+      <c r="E25" s="3"/>
+      <c r="F25" s="3"/>
+      <c r="G25" s="3"/>
+      <c r="H25" s="3"/>
+      <c r="I25" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="J25" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="K25" s="3" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="B26" s="3"/>
+      <c r="C26" s="3"/>
+      <c r="D26" s="3"/>
+      <c r="E26" s="3"/>
+      <c r="F26" s="3"/>
+      <c r="G26" s="3"/>
+      <c r="H26" s="3"/>
+      <c r="I26" s="3"/>
+      <c r="J26" s="3"/>
+      <c r="K26" s="3" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="B27" s="3"/>
+      <c r="C27" s="3"/>
+      <c r="D27" s="3"/>
+      <c r="E27" s="3"/>
+      <c r="F27" s="3"/>
+      <c r="G27" s="3"/>
+      <c r="H27" s="3"/>
+      <c r="I27" s="3"/>
+      <c r="J27" s="3"/>
+      <c r="K27" s="3" t="s">
+        <v>12</v>
+      </c>
+    </row>
     <row r="28" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="29" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="30" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>

</xml_diff>